<commit_message>
Current progress and fix on deliveryagreement
</commit_message>
<xml_diff>
--- a/Vorlagen/Ablieferungsverzeichnis, Vorlage.xlsx
+++ b/Vorlagen/Ablieferungsverzeichnis, Vorlage.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\home.kt.ktzh.ch\BAA7556$\Desktop\Projects\delivery-macro\Vorlagen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD0D1795-31D4-45E7-8928-192FEEE3A38A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{651E8754-CC94-42EB-87FF-8BE0B31B687D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
   <si>
     <t>Menge</t>
   </si>
@@ -146,6 +146,9 @@
       </rPr>
       <t xml:space="preserve"> (z.B. 3 Ordner, 10 Schachteln, 50 PDF-Dateien)</t>
     </r>
+  </si>
+  <si>
+    <t>&lt;AblNummer&gt;</t>
   </si>
 </sst>
 </file>
@@ -929,7 +932,9 @@
       <c r="B19" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C19" s="5"/>
+      <c r="C19" s="6" t="s">
+        <v>23</v>
+      </c>
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
       <c r="F19" s="3"/>

</xml_diff>